<commit_message>
update ota-driver for 9.0
</commit_message>
<xml_diff>
--- a/ota-driver/pkg/ota/resources/findings.xlsx
+++ b/ota-driver/pkg/ota/resources/findings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALAINRobert\Documents\Dvlpt\support\onprem\advisor\odm-transformation-advisor\ota-bom\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dvlpt\odm-transformation-advisor\ota-bom\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A9B0E81-F203-405A-9988-6D2E54DCD1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F39BD5-5B65-4F73-BE50-0CE6788CFCEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3200" yWindow="3280" windowWidth="22310" windowHeight="12250" tabRatio="314" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="62700" yWindow="1965" windowWidth="23280" windowHeight="14610" tabRatio="314" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="findings" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="222">
   <si>
     <t>CLASSIC_PROJECT</t>
   </si>
@@ -556,9 +556,6 @@
     <t>Classic rule projects removed</t>
   </si>
   <si>
-    <t>Some rule projects are organized using Classic Rule Projects (see your project &lt;em&gt;%2$s&lt;/em&gt;, for example). Classic Rule Projects are removed since ODM version 8.11.0. It is recommended that you migrate to projects organized as &lt;em&gt;Decision Services&lt;/em&gt;. ODM provides an automated migration tool that will help you perform that project migration.&lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurence%4$s found&lt;/b&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">decision  model </t>
   </si>
   <si>
@@ -598,9 +595,6 @@
     <t>return "TEMPLATE_REMOVED";</t>
   </si>
   <si>
-    <t>Ruleset Without Ruleflow</t>
-  </si>
-  <si>
     <t>RULESET_WITHOUT_RULEFLOW</t>
   </si>
   <si>
@@ -643,9 +637,6 @@
     <t>The use of operation without a ruleflow is deprecated since ODM 8.12.0. It is recommended to create  a ruleflow with a RETE task instead. &lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurrence%4$s found&lt;/b&gt;</t>
   </si>
   <si>
-    <t>The use of the Classic Rule Engine (CRE)  was detected in some of the rule projects (see your project &lt;em&gt;%2$s&lt;/em&gt;, for example). The CRE is removed since ODM version 8.12.0. Migration to the more efficient Decision Engine is recommended.&lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurence%4$s found&lt;/b&gt;</t>
-  </si>
-  <si>
     <t>Some projects are using custom rule languages that are no longer supported since 8.11.&lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurence%4$s found&lt;/b&gt;</t>
   </si>
   <si>
@@ -656,6 +647,60 @@
   </si>
   <si>
     <t>return "RULESET_WITHOUT_RULEFLOW";</t>
+  </si>
+  <si>
+    <t>XML_BINDING</t>
+  </si>
+  <si>
+    <t>XML Binding usage</t>
+  </si>
+  <si>
+    <t>XOM Management not enabled</t>
+  </si>
+  <si>
+    <t>XOM_MANAGEMENT_IN_DC</t>
+  </si>
+  <si>
+    <t>return "XOM_MANAGEMENT_IN_DC";</t>
+  </si>
+  <si>
+    <t>XOM Management</t>
+  </si>
+  <si>
+    <t>XML Binding</t>
+  </si>
+  <si>
+    <t>return "XML_BINDING";</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>&amp;#128505</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>Compatible</t>
+  </si>
+  <si>
+    <t>Not Compatible</t>
+  </si>
+  <si>
+    <t>The use of the Classic Rule Engine (CRE)  was detected in some of the rule projects (see your project &lt;em&gt;%1$s&lt;/em&gt;, for example). The CRE is removed since ODM version 8.12.0. Migration to the more efficient Decision Engine is recommended.&lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurence%4$s found&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Some decision service do not use XOM management in DC. This is deprecated in 9.0 (see your project &lt;em&gt;%1$s&lt;/em&gt;).&lt;br&gt;It is recommended to enable XOM management in Rule Designer and update project in Decision Center. &lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurence%4$s found&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Some rule projects are organized using Classic Rule Projects (see your project &lt;em&gt;%1$s&lt;/em&gt;, for example). Classic Rule Projects are removed since ODM version 8.11.0. It is recommended that you migrate to projects organized as &lt;em&gt;Decision Services&lt;/em&gt;. ODM provides an automated migration tool that will help you perform that project migration.&lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurence%4$s found&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Some decision service use XML Binding. This is deprecated in 8.11.1 (see your project &lt;em&gt;%1$s&lt;/em&gt;).&lt;br&gt;It is recommended to replace XML Binding with a java XOM generated from JAXB for example. &lt;br&gt;&lt;br&gt;&lt;b&gt;%3$s occurence%4$s found&lt;/b&gt;</t>
   </si>
 </sst>
 </file>
@@ -834,7 +879,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -891,7 +936,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1172,7 +1217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.7265625" style="1" bestFit="1" customWidth="1"/>
@@ -1283,7 +1328,7 @@
         <v>133</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
@@ -1872,16 +1917,16 @@
         <v>172</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>173</v>
+        <v>220</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>170</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>133</v>
@@ -1890,46 +1935,46 @@
     </row>
     <row r="30" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>133</v>
       </c>
       <c r="H30" s="11"/>
     </row>
-    <row r="31" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>176</v>
-      </c>
       <c r="C31" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>170</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>133</v>
@@ -1938,22 +1983,22 @@
     </row>
     <row r="32" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>180</v>
-      </c>
       <c r="C32" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>170</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>133</v>
@@ -1962,22 +2007,22 @@
     </row>
     <row r="33" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>170</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G33" s="12" t="s">
         <v>133</v>
@@ -1986,22 +2031,22 @@
     </row>
     <row r="34" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>170</v>
       </c>
       <c r="E34" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>185</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>186</v>
       </c>
       <c r="G34" s="12" t="s">
         <v>133</v>
@@ -2010,24 +2055,70 @@
     </row>
     <row r="35" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>187</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F35" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="69.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="F36" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>133</v>
       </c>
     </row>
@@ -2040,7 +2131,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
@@ -2080,7 +2171,7 @@
         <v>63</v>
       </c>
       <c r="E2" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2114,7 +2205,7 @@
         <v>134</v>
       </c>
       <c r="E4" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -2125,13 +2216,47 @@
         <v>169</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E5" s="24">
-        <v>3</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="24" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>214</v>
+      </c>
+      <c r="E6" s="24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>198</v>
+      </c>
+      <c r="E7" s="24">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>